<commit_message>
test: regenerate golden snapshots and the reference template with charts (#131)
The three spreading snapshots gain only chart serialization lines --
every cell, formula and figure line is byte-for-byte unchanged (the
diff adds lines, deletes none). The framework-computed fixture's series
extends to column H because its downside covers FY+1 alone; the blank
and analyst-supplied cases stay on B..G.

The reference template is regenerated with its documented command
(templates/README.md), which now also carries the two charts. It had
silently drifted: its last regeneration (9d0f9f8) predates the
issue-169 IF-guarded ratio formulas and the issue-99 working-capital
formulas, so the regeneration brings those columns' formulas in line
with the current builder output that spreading_blank.xlsx.txt already
pins -- the normalized template is byte-identical to that snapshot.
</commit_message>
<xml_diff>
--- a/templates/spreading/default_spreading_template.xlsx
+++ b/templates/spreading/default_spreading_template.xlsx
@@ -132,6 +132,257 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Leverage Trend</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <lineChart>
+        <grouping val="standard"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Financial Spreading'!$A$58</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Financial Spreading'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Financial Spreading'!$B$58:$G$58</f>
+            </numRef>
+          </val>
+        </ser>
+        <ser>
+          <idx val="1"/>
+          <order val="1"/>
+          <tx>
+            <strRef>
+              <f>'Financial Spreading'!$A$59</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <marker>
+            <symbol val="none"/>
+            <spPr>
+              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+                <a:prstDash val="solid"/>
+              </a:ln>
+            </spPr>
+          </marker>
+          <cat>
+            <numRef>
+              <f>'Financial Spreading'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Financial Spreading'!$B$59:$G$59</f>
+            </numRef>
+          </val>
+        </ser>
+        <axId val="10"/>
+        <axId val="100"/>
+      </lineChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/charts/chart2.xml><?xml version="1.0" encoding="utf-8"?>
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+  <chart>
+    <title>
+      <tx>
+        <rich>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:pPr>
+              <a:defRPr/>
+            </a:pPr>
+            <a:r>
+              <a:t>Revenue Trend</a:t>
+            </a:r>
+          </a:p>
+        </rich>
+      </tx>
+    </title>
+    <plotArea>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <ser>
+          <idx val="0"/>
+          <order val="0"/>
+          <tx>
+            <strRef>
+              <f>'Financial Spreading'!$A$3</f>
+            </strRef>
+          </tx>
+          <spPr>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:prstDash val="solid"/>
+            </a:ln>
+          </spPr>
+          <cat>
+            <numRef>
+              <f>'Financial Spreading'!$B$1:$G$1</f>
+            </numRef>
+          </cat>
+          <val>
+            <numRef>
+              <f>'Financial Spreading'!$B$3:$G$3</f>
+            </numRef>
+          </val>
+        </ser>
+        <gapWidth val="150"/>
+        <axId val="10"/>
+        <axId val="100"/>
+      </barChart>
+      <catAx>
+        <axId val="10"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="100"/>
+        <lblOffset val="100"/>
+      </catAx>
+      <valAx>
+        <axId val="100"/>
+        <scaling>
+          <orientation val="minMax"/>
+        </scaling>
+        <axPos val="l"/>
+        <majorGridlines/>
+        <majorTickMark val="none"/>
+        <minorTickMark val="none"/>
+        <crossAx val="10"/>
+      </valAx>
+    </plotArea>
+    <legend>
+      <legendPos val="r"/>
+    </legend>
+    <plotVisOnly val="1"/>
+    <dispBlanksAs val="gap"/>
+  </chart>
+</chartSpace>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>65</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="1" name="Chart 1"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>83</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="5400000" cy="2700000"/>
+    <graphicFrame>
+      <nvGraphicFramePr>
+        <cNvPr id="2" name="Chart 2"/>
+        <cNvGraphicFramePr/>
+      </nvGraphicFramePr>
+      <xfrm/>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+        </a:graphicData>
+      </a:graphic>
+    </graphicFrame>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -561,39 +812,39 @@
         </is>
       </c>
       <c r="B6">
-        <f>IFERROR(B5/B3,"N/A")</f>
+        <f>IFERROR(IF((B3)&gt;0,(B5)/(B3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C6">
-        <f>IFERROR(C5/C3,"N/A")</f>
+        <f>IFERROR(IF((C3)&gt;0,(C5)/(C3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D6">
-        <f>IFERROR(D5/D3,"N/A")</f>
+        <f>IFERROR(IF((D3)&gt;0,(D5)/(D3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E6">
-        <f>IFERROR(E5/E3,"N/A")</f>
+        <f>IFERROR(IF((E3)&gt;0,(E5)/(E3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F6">
-        <f>IFERROR(F5/F3,"N/A")</f>
+        <f>IFERROR(IF((F3)&gt;0,(F5)/(F3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G6">
-        <f>IFERROR(G5/G3,"N/A")</f>
+        <f>IFERROR(IF((G3)&gt;0,(G5)/(G3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H6">
-        <f>IFERROR(H5/H3,"N/A")</f>
+        <f>IFERROR(IF((H3)&gt;0,(H5)/(H3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I6">
-        <f>IFERROR(I5/I3,"N/A")</f>
+        <f>IFERROR(IF((I3)&gt;0,(I5)/(I3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J6">
-        <f>IFERROR(J5/J3,"N/A")</f>
+        <f>IFERROR(IF((J3)&gt;0,(J5)/(J3),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -675,39 +926,39 @@
         </is>
       </c>
       <c r="B12">
-        <f>IFERROR(B11/B3,"N/A")</f>
+        <f>IFERROR(IF((B3)&gt;0,(B11)/(B3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C12">
-        <f>IFERROR(C11/C3,"N/A")</f>
+        <f>IFERROR(IF((C3)&gt;0,(C11)/(C3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D12">
-        <f>IFERROR(D11/D3,"N/A")</f>
+        <f>IFERROR(IF((D3)&gt;0,(D11)/(D3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E12">
-        <f>IFERROR(E11/E3,"N/A")</f>
+        <f>IFERROR(IF((E3)&gt;0,(E11)/(E3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F12">
-        <f>IFERROR(F11/F3,"N/A")</f>
+        <f>IFERROR(IF((F3)&gt;0,(F11)/(F3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G12">
-        <f>IFERROR(G11/G3,"N/A")</f>
+        <f>IFERROR(IF((G3)&gt;0,(G11)/(G3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H12">
-        <f>IFERROR(H11/H3,"N/A")</f>
+        <f>IFERROR(IF((H3)&gt;0,(H11)/(H3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I12">
-        <f>IFERROR(I11/I3,"N/A")</f>
+        <f>IFERROR(IF((I3)&gt;0,(I11)/(I3),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J12">
-        <f>IFERROR(J11/J3,"N/A")</f>
+        <f>IFERROR(IF((J3)&gt;0,(J11)/(J3),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -896,39 +1147,39 @@
         </is>
       </c>
       <c r="B23">
-        <f>IFERROR(B13/(B14+B16),"N/A")</f>
+        <f>IFERROR(IF((B14+B16)&gt;0,(B13)/(B14+B16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C23">
-        <f>IFERROR(C13/(C14+C16),"N/A")</f>
+        <f>IFERROR(IF((C14+C16)&gt;0,(C13)/(C14+C16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D23">
-        <f>IFERROR(D13/(D14+D16),"N/A")</f>
+        <f>IFERROR(IF((D14+D16)&gt;0,(D13)/(D14+D16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E23">
-        <f>IFERROR(E13/(E14+E16),"N/A")</f>
+        <f>IFERROR(IF((E14+E16)&gt;0,(E13)/(E14+E16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F23">
-        <f>IFERROR(F13/(F14+F16),"N/A")</f>
+        <f>IFERROR(IF((F14+F16)&gt;0,(F13)/(F14+F16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G23">
-        <f>IFERROR(G13/(G14+G16),"N/A")</f>
+        <f>IFERROR(IF((G14+G16)&gt;0,(G13)/(G14+G16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H23">
-        <f>IFERROR(H13/(H14+H16),"N/A")</f>
+        <f>IFERROR(IF((H14+H16)&gt;0,(H13)/(H14+H16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I23">
-        <f>IFERROR(I13/(I14+I16),"N/A")</f>
+        <f>IFERROR(IF((I14+I16)&gt;0,(I13)/(I14+I16),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J23">
-        <f>IFERROR(J13/(J14+J16),"N/A")</f>
+        <f>IFERROR(IF((J14+J16)&gt;0,(J13)/(J14+J16),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -939,39 +1190,39 @@
         </is>
       </c>
       <c r="B24">
-        <f>IFERROR(B11/B14,"N/A")</f>
+        <f>IFERROR(IF((B14)&gt;0,(B11)/(B14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C24">
-        <f>IFERROR(C11/C14,"N/A")</f>
+        <f>IFERROR(IF((C14)&gt;0,(C11)/(C14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D24">
-        <f>IFERROR(D11/D14,"N/A")</f>
+        <f>IFERROR(IF((D14)&gt;0,(D11)/(D14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E24">
-        <f>IFERROR(E11/E14,"N/A")</f>
+        <f>IFERROR(IF((E14)&gt;0,(E11)/(E14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F24">
-        <f>IFERROR(F11/F14,"N/A")</f>
+        <f>IFERROR(IF((F14)&gt;0,(F11)/(F14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G24">
-        <f>IFERROR(G11/G14,"N/A")</f>
+        <f>IFERROR(IF((G14)&gt;0,(G11)/(G14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H24">
-        <f>IFERROR(H11/H14,"N/A")</f>
+        <f>IFERROR(IF((H14)&gt;0,(H11)/(H14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I24">
-        <f>IFERROR(I11/I14,"N/A")</f>
+        <f>IFERROR(IF((I14)&gt;0,(I11)/(I14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J24">
-        <f>IFERROR(J11/J14,"N/A")</f>
+        <f>IFERROR(IF((J14)&gt;0,(J11)/(J14),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -982,39 +1233,39 @@
         </is>
       </c>
       <c r="B25">
-        <f>IFERROR(B13/B14,"N/A")</f>
+        <f>IFERROR(IF((B14)&gt;0,(B13)/(B14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C25">
-        <f>IFERROR(C13/C14,"N/A")</f>
+        <f>IFERROR(IF((C14)&gt;0,(C13)/(C14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D25">
-        <f>IFERROR(D13/D14,"N/A")</f>
+        <f>IFERROR(IF((D14)&gt;0,(D13)/(D14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E25">
-        <f>IFERROR(E13/E14,"N/A")</f>
+        <f>IFERROR(IF((E14)&gt;0,(E13)/(E14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F25">
-        <f>IFERROR(F13/F14,"N/A")</f>
+        <f>IFERROR(IF((F14)&gt;0,(F13)/(F14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G25">
-        <f>IFERROR(G13/G14,"N/A")</f>
+        <f>IFERROR(IF((G14)&gt;0,(G13)/(G14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H25">
-        <f>IFERROR(H13/H14,"N/A")</f>
+        <f>IFERROR(IF((H14)&gt;0,(H13)/(H14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I25">
-        <f>IFERROR(I13/I14,"N/A")</f>
+        <f>IFERROR(IF((I14)&gt;0,(I13)/(I14),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J25">
-        <f>IFERROR(J13/J14,"N/A")</f>
+        <f>IFERROR(IF((J14)&gt;0,(J13)/(J14),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1068,39 +1319,39 @@
         </is>
       </c>
       <c r="B27">
-        <f>IFERROR(B26/B13,"N/A")</f>
+        <f>IFERROR(IF((B13)&gt;0,(B26)/(B13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C27">
-        <f>IFERROR(C26/C13,"N/A")</f>
+        <f>IFERROR(IF((C13)&gt;0,(C26)/(C13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D27">
-        <f>IFERROR(D26/D13,"N/A")</f>
+        <f>IFERROR(IF((D13)&gt;0,(D26)/(D13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E27">
-        <f>IFERROR(E26/E13,"N/A")</f>
+        <f>IFERROR(IF((E13)&gt;0,(E26)/(E13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F27">
-        <f>IFERROR(F26/F13,"N/A")</f>
+        <f>IFERROR(IF((F13)&gt;0,(F26)/(F13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G27">
-        <f>IFERROR(G26/G13,"N/A")</f>
+        <f>IFERROR(IF((G13)&gt;0,(G26)/(G13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H27">
-        <f>IFERROR(H26/H13,"N/A")</f>
+        <f>IFERROR(IF((H13)&gt;0,(H26)/(H13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I27">
-        <f>IFERROR(I26/I13,"N/A")</f>
+        <f>IFERROR(IF((I13)&gt;0,(I26)/(I13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J27">
-        <f>IFERROR(J26/J13,"N/A")</f>
+        <f>IFERROR(IF((J13)&gt;0,(J26)/(J13),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1631,39 +1882,39 @@
         </is>
       </c>
       <c r="B56">
-        <f>IFERROR((B40+B41+B44+B45)/B52,"N/A")</f>
+        <f>IFERROR(IF((B52)&gt;0,(B40+B41+B44+B45)/(B52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C56">
-        <f>IFERROR((C40+C41+C44+C45)/C52,"N/A")</f>
+        <f>IFERROR(IF((C52)&gt;0,(C40+C41+C44+C45)/(C52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D56">
-        <f>IFERROR((D40+D41+D44+D45)/D52,"N/A")</f>
+        <f>IFERROR(IF((D52)&gt;0,(D40+D41+D44+D45)/(D52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E56">
-        <f>IFERROR((E40+E41+E44+E45)/E52,"N/A")</f>
+        <f>IFERROR(IF((E52)&gt;0,(E40+E41+E44+E45)/(E52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F56">
-        <f>IFERROR((F40+F41+F44+F45)/F52,"N/A")</f>
+        <f>IFERROR(IF((F52)&gt;0,(F40+F41+F44+F45)/(F52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G56">
-        <f>IFERROR((G40+G41+G44+G45)/G52,"N/A")</f>
+        <f>IFERROR(IF((G52)&gt;0,(G40+G41+G44+G45)/(G52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H56">
-        <f>IFERROR((H40+H41+H44+H45)/H52,"N/A")</f>
+        <f>IFERROR(IF((H52)&gt;0,(H40+H41+H44+H45)/(H52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I56">
-        <f>IFERROR((I40+I41+I44+I45)/I52,"N/A")</f>
+        <f>IFERROR(IF((I52)&gt;0,(I40+I41+I44+I45)/(I52),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J56">
-        <f>IFERROR((J40+J41+J44+J45)/J52,"N/A")</f>
+        <f>IFERROR(IF((J52)&gt;0,(J40+J41+J44+J45)/(J52),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1674,39 +1925,39 @@
         </is>
       </c>
       <c r="B57">
-        <f>IFERROR(B37/B43,"N/A")</f>
+        <f>IFERROR(IF((B43)&gt;0,(B37)/(B43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C57">
-        <f>IFERROR(C37/C43,"N/A")</f>
+        <f>IFERROR(IF((C43)&gt;0,(C37)/(C43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D57">
-        <f>IFERROR(D37/D43,"N/A")</f>
+        <f>IFERROR(IF((D43)&gt;0,(D37)/(D43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E57">
-        <f>IFERROR(E37/E43,"N/A")</f>
+        <f>IFERROR(IF((E43)&gt;0,(E37)/(E43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F57">
-        <f>IFERROR(F37/F43,"N/A")</f>
+        <f>IFERROR(IF((F43)&gt;0,(F37)/(F43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G57">
-        <f>IFERROR(G37/G43,"N/A")</f>
+        <f>IFERROR(IF((G43)&gt;0,(G37)/(G43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H57">
-        <f>IFERROR(H37/H43,"N/A")</f>
+        <f>IFERROR(IF((H43)&gt;0,(H37)/(H43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I57">
-        <f>IFERROR(I37/I43,"N/A")</f>
+        <f>IFERROR(IF((I43)&gt;0,(I37)/(I43),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J57">
-        <f>IFERROR(J37/J43,"N/A")</f>
+        <f>IFERROR(IF((J43)&gt;0,(J37)/(J43),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1717,39 +1968,39 @@
         </is>
       </c>
       <c r="B58">
-        <f>IFERROR((B40+B41+B44+B45)/B13,"N/A")</f>
+        <f>IFERROR(IF((B13)&gt;0,(B40+B41+B44+B45)/(B13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C58">
-        <f>IFERROR((C40+C41+C44+C45)/C13,"N/A")</f>
+        <f>IFERROR(IF((C13)&gt;0,(C40+C41+C44+C45)/(C13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D58">
-        <f>IFERROR((D40+D41+D44+D45)/D13,"N/A")</f>
+        <f>IFERROR(IF((D13)&gt;0,(D40+D41+D44+D45)/(D13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E58">
-        <f>IFERROR((E40+E41+E44+E45)/E13,"N/A")</f>
+        <f>IFERROR(IF((E13)&gt;0,(E40+E41+E44+E45)/(E13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F58">
-        <f>IFERROR((F40+F41+F44+F45)/F13,"N/A")</f>
+        <f>IFERROR(IF((F13)&gt;0,(F40+F41+F44+F45)/(F13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G58">
-        <f>IFERROR((G40+G41+G44+G45)/G13,"N/A")</f>
+        <f>IFERROR(IF((G13)&gt;0,(G40+G41+G44+G45)/(G13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H58">
-        <f>IFERROR((H40+H41+H44+H45)/H13,"N/A")</f>
+        <f>IFERROR(IF((H13)&gt;0,(H40+H41+H44+H45)/(H13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I58">
-        <f>IFERROR((I40+I41+I44+I45)/I13,"N/A")</f>
+        <f>IFERROR(IF((I13)&gt;0,(I40+I41+I44+I45)/(I13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J58">
-        <f>IFERROR((J40+J41+J44+J45)/J13,"N/A")</f>
+        <f>IFERROR(IF((J13)&gt;0,(J40+J41+J44+J45)/(J13),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1760,39 +2011,39 @@
         </is>
       </c>
       <c r="B59">
-        <f>IFERROR((B40+B41+B44+B45-B33)/B13,"N/A")</f>
+        <f>IFERROR(IF((B13)&gt;0,(B40+B41+B44+B45-B33)/(B13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="C59">
-        <f>IFERROR((C40+C41+C44+C45-C33)/C13,"N/A")</f>
+        <f>IFERROR(IF((C13)&gt;0,(C40+C41+C44+C45-C33)/(C13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="D59">
-        <f>IFERROR((D40+D41+D44+D45-D33)/D13,"N/A")</f>
+        <f>IFERROR(IF((D13)&gt;0,(D40+D41+D44+D45-D33)/(D13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="E59">
-        <f>IFERROR((E40+E41+E44+E45-E33)/E13,"N/A")</f>
+        <f>IFERROR(IF((E13)&gt;0,(E40+E41+E44+E45-E33)/(E13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="F59">
-        <f>IFERROR((F40+F41+F44+F45-F33)/F13,"N/A")</f>
+        <f>IFERROR(IF((F13)&gt;0,(F40+F41+F44+F45-F33)/(F13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="G59">
-        <f>IFERROR((G40+G41+G44+G45-G33)/G13,"N/A")</f>
+        <f>IFERROR(IF((G13)&gt;0,(G40+G41+G44+G45-G33)/(G13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="H59">
-        <f>IFERROR((H40+H41+H44+H45-H33)/H13,"N/A")</f>
+        <f>IFERROR(IF((H13)&gt;0,(H40+H41+H44+H45-H33)/(H13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="I59">
-        <f>IFERROR((I40+I41+I44+I45-I33)/I13,"N/A")</f>
+        <f>IFERROR(IF((I13)&gt;0,(I40+I41+I44+I45-I33)/(I13),"N/A"),"N/A")</f>
         <v/>
       </c>
       <c r="J59">
-        <f>IFERROR((J40+J41+J44+J45-J33)/J13,"N/A")</f>
+        <f>IFERROR(IF((J13)&gt;0,(J40+J41+J44+J45-J33)/(J13),"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -1809,6 +2060,42 @@
           <t>Trade Debtor Days</t>
         </is>
       </c>
+      <c r="B61">
+        <f>IFERROR(IF((B3)&gt;0,(B34)/(B3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="C61">
+        <f>IFERROR(IF((C3)&gt;0,(C34)/(C3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="D61">
+        <f>IFERROR(IF((D3)&gt;0,(D34)/(D3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="E61">
+        <f>IFERROR(IF((E3)&gt;0,(E34)/(E3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F61">
+        <f>IFERROR(IF((F3)&gt;0,(F34)/(F3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="G61">
+        <f>IFERROR(IF((G3)&gt;0,(G34)/(G3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="H61">
+        <f>IFERROR(IF((H3)&gt;0,(H34)/(H3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="I61">
+        <f>IFERROR(IF((I3)&gt;0,(I34)/(I3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="J61">
+        <f>IFERROR(IF((J3)&gt;0,(J34)/(J3)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1816,6 +2103,42 @@
           <t>Trade Creditor Days</t>
         </is>
       </c>
+      <c r="B62">
+        <f>IFERROR(IF((B4)&gt;0,(B39)/(B4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="C62">
+        <f>IFERROR(IF((C4)&gt;0,(C39)/(C4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="D62">
+        <f>IFERROR(IF((D4)&gt;0,(D39)/(D4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="E62">
+        <f>IFERROR(IF((E4)&gt;0,(E39)/(E4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F62">
+        <f>IFERROR(IF((F4)&gt;0,(F39)/(F4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="G62">
+        <f>IFERROR(IF((G4)&gt;0,(G39)/(G4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="H62">
+        <f>IFERROR(IF((H4)&gt;0,(H39)/(H4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="I62">
+        <f>IFERROR(IF((I4)&gt;0,(I39)/(I4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="J62">
+        <f>IFERROR(IF((J4)&gt;0,(J39)/(J4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1823,6 +2146,42 @@
           <t>Stock Days</t>
         </is>
       </c>
+      <c r="B63">
+        <f>IFERROR(IF((B4)&gt;0,(B35)/(B4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="C63">
+        <f>IFERROR(IF((C4)&gt;0,(C35)/(C4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="D63">
+        <f>IFERROR(IF((D4)&gt;0,(D35)/(D4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="E63">
+        <f>IFERROR(IF((E4)&gt;0,(E35)/(E4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="F63">
+        <f>IFERROR(IF((F4)&gt;0,(F35)/(F4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="G63">
+        <f>IFERROR(IF((G4)&gt;0,(G35)/(G4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="H63">
+        <f>IFERROR(IF((H4)&gt;0,(H35)/(H4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="I63">
+        <f>IFERROR(IF((I4)&gt;0,(I35)/(I4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
+      <c r="J63">
+        <f>IFERROR(IF((J4)&gt;0,(J35)/(J4)*365,"N/A"),"N/A")</f>
+        <v/>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1831,44 +2190,45 @@
         </is>
       </c>
       <c r="B64">
-        <f>B61+B63-B62</f>
+        <f>IFERROR(B61+B63-B62,"N/A")</f>
         <v/>
       </c>
       <c r="C64">
-        <f>C61+C63-C62</f>
+        <f>IFERROR(C61+C63-C62,"N/A")</f>
         <v/>
       </c>
       <c r="D64">
-        <f>D61+D63-D62</f>
+        <f>IFERROR(D61+D63-D62,"N/A")</f>
         <v/>
       </c>
       <c r="E64">
-        <f>E61+E63-E62</f>
+        <f>IFERROR(E61+E63-E62,"N/A")</f>
         <v/>
       </c>
       <c r="F64">
-        <f>F61+F63-F62</f>
+        <f>IFERROR(F61+F63-F62,"N/A")</f>
         <v/>
       </c>
       <c r="G64">
-        <f>G61+G63-G62</f>
+        <f>IFERROR(G61+G63-G62,"N/A")</f>
         <v/>
       </c>
       <c r="H64">
-        <f>H61+H63-H62</f>
+        <f>IFERROR(H61+H63-H62,"N/A")</f>
         <v/>
       </c>
       <c r="I64">
-        <f>I61+I63-I62</f>
+        <f>IFERROR(I61+I63-I62,"N/A")</f>
         <v/>
       </c>
       <c r="J64">
-        <f>J61+J63-J62</f>
+        <f>IFERROR(J61+J63-J62,"N/A")</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
docs+test: describe the base-case and downside chart layout; regenerate snapshot and template (#131, D1)
The snapshot diff is chart lines only (B-G ranges, one new downside chart); the template
is regenerated with the documented command so it carries #371's collateral formulas and the charts.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01PUGYmUgRq5YEtDPW9fVgJy
</commit_message>
<xml_diff>
--- a/templates/spreading/default_spreading_template.xlsx
+++ b/templates/spreading/default_spreading_template.xlsx
@@ -2301,7 +2301,7 @@
     </row>
     <row r="2">
       <c r="H2">
-        <f>IFERROR(G2/B2,"N/A")</f>
+        <f>IFERROR(IF(B2&gt;0,G2/B2,"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>
@@ -2336,7 +2336,7 @@
         <v/>
       </c>
       <c r="H3">
-        <f>IFERROR(G3/B3,"N/A")</f>
+        <f>IFERROR(IF(B3&gt;0,G3/B3,"N/A"),"N/A")</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
fix: make all three spreading charts clustered columns with visible axes
The maintainer's manual Excel check (issue #131, comment 6277984249) found
that a line chart plots a text N/A cell as zero, that openpyxl 3.1+
writes axes as deleted unless delete=False, and that a single-series bar
chart with varyColors unset gives one colour per period (a period
legend). Implement option A (comment 6278038868): the leverage, revenue
and downside charts are all clustered column charts, both axes of every
chart are explicitly not deleted, and varyColors is off so the legend
names the series. Chart titles and anchors are unchanged; no cell,
formula or figure changes (the regenerated snapshots differ only in the
four chart-type lines; every cell line is byte-identical). Correct the
_write_charts docstring and the docs/outputs.md paragraphs: a text N/A
draws as an empty slot, a true blank as a gap, neither as zero.
</commit_message>
<xml_diff>
--- a/templates/spreading/default_spreading_template.xlsx
+++ b/templates/spreading/default_spreading_template.xlsx
@@ -153,8 +153,10 @@
       </tx>
     </title>
     <plotArea>
-      <lineChart>
-        <grouping val="standard"/>
+      <barChart>
+        <barDir val="col"/>
+        <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -168,14 +170,6 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
               <f>'Financial Spreading'!$B$1:$G$1</f>
@@ -200,14 +194,6 @@
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
-          <marker>
-            <symbol val="none"/>
-            <spPr>
-              <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-                <a:prstDash val="solid"/>
-              </a:ln>
-            </spPr>
-          </marker>
           <cat>
             <numRef>
               <f>'Financial Spreading'!$B$1:$G$1</f>
@@ -219,14 +205,16 @@
             </numRef>
           </val>
         </ser>
+        <gapWidth val="150"/>
         <axId val="10"/>
         <axId val="100"/>
-      </lineChart>
+      </barChart>
       <catAx>
         <axId val="10"/>
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -238,6 +226,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <majorTickMark val="none"/>
@@ -276,6 +265,7 @@
       <barChart>
         <barDir val="col"/>
         <grouping val="clustered"/>
+        <varyColors val="0"/>
         <ser>
           <idx val="0"/>
           <order val="0"/>
@@ -309,6 +299,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
@@ -320,6 +311,7 @@
         <scaling>
           <orientation val="minMax"/>
         </scaling>
+        <delete val="0"/>
         <axPos val="l"/>
         <majorGridlines/>
         <majorTickMark val="none"/>

</xml_diff>